<commit_message>
Added a new row to the Excel file
</commit_message>
<xml_diff>
--- a/Price Data.xlsx
+++ b/Price Data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E343"/>
+  <dimension ref="A1:E344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6537,6 +6537,25 @@
         <v>6.9639</v>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-03-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="B344" t="n">
+        <v>155500</v>
+      </c>
+      <c r="C344" t="n">
+        <v>22537.21</v>
+      </c>
+      <c r="D344" t="n">
+        <v>19944.44</v>
+      </c>
+      <c r="E344" t="n">
+        <v>6.8728</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>